<commit_message>
ARR analytics updated Mar
</commit_message>
<xml_diff>
--- a/backend/data/closed_acv.xlsx
+++ b/backend/data/closed_acv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gep1-my.sharepoint.com/personal/ajoseph_gep_com/Documents/Desktop/Project-Aether-Enterprise/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="147" documentId="8_{E886ED90-0776-4F81-A4C1-54B160D1665C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53F42021-D1B9-4948-BEEF-0D806D122B17}"/>
+  <xr:revisionPtr revIDLastSave="166" documentId="8_{E886ED90-0776-4F81-A4C1-54B160D1665C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B07EDD5A-B696-4406-9D7B-BC8D9F77B9DD}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{362E1928-A501-4CAC-8243-2F29D3895462}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4931" uniqueCount="1399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4931" uniqueCount="1397">
   <si>
     <t>Closed_ACV_ID</t>
   </si>
@@ -4224,12 +4224,6 @@
   </si>
   <si>
     <t>Logitech Europe S.A</t>
-  </si>
-  <si>
-    <t>CrossSell</t>
-  </si>
-  <si>
-    <t>New</t>
   </si>
   <si>
     <t>Johnson Fernandez</t>
@@ -5132,6 +5126,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19" customWidth="1"/>
     <col min="18" max="18" width="18.90625" bestFit="1" customWidth="1"/>
   </cols>
@@ -17049,7 +17044,7 @@
         <v>155000</v>
       </c>
       <c r="O297" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
       <c r="P297">
         <v>3337</v>
@@ -17087,7 +17082,7 @@
         <v>165000</v>
       </c>
       <c r="O298" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
       <c r="P298">
         <v>3338</v>
@@ -28985,7 +28980,7 @@
       <c r="E597" s="1">
         <v>46023</v>
       </c>
-      <c r="F597" s="6" t="s">
+      <c r="F597" t="s">
         <v>34</v>
       </c>
       <c r="G597" t="s">
@@ -29150,7 +29145,7 @@
         <v>850000</v>
       </c>
       <c r="O601" s="6" t="s">
-        <v>1397</v>
+        <v>1395</v>
       </c>
       <c r="P601">
         <v>1327</v>
@@ -29178,8 +29173,8 @@
       <c r="E602" s="1">
         <v>46054</v>
       </c>
-      <c r="F602" s="6" t="s">
-        <v>1395</v>
+      <c r="F602" t="s">
+        <v>126</v>
       </c>
       <c r="G602" t="s">
         <v>40</v>
@@ -29219,8 +29214,8 @@
       <c r="E603" s="1">
         <v>46054</v>
       </c>
-      <c r="F603" s="6" t="s">
-        <v>1395</v>
+      <c r="F603" t="s">
+        <v>126</v>
       </c>
       <c r="G603" t="s">
         <v>22</v>
@@ -29260,8 +29255,8 @@
       <c r="E604" s="1">
         <v>46054</v>
       </c>
-      <c r="F604" s="6" t="s">
-        <v>1396</v>
+      <c r="F604" t="s">
+        <v>34</v>
       </c>
       <c r="G604" t="s">
         <v>40</v>
@@ -29301,8 +29296,8 @@
       <c r="E605" s="1">
         <v>46054</v>
       </c>
-      <c r="F605" s="6" t="s">
-        <v>1396</v>
+      <c r="F605" t="s">
+        <v>34</v>
       </c>
       <c r="G605" t="s">
         <v>22</v>
@@ -29342,8 +29337,8 @@
       <c r="E606" s="1">
         <v>46054</v>
       </c>
-      <c r="F606" s="6" t="s">
-        <v>1396</v>
+      <c r="F606" t="s">
+        <v>34</v>
       </c>
       <c r="G606" t="s">
         <v>22</v>
@@ -29383,8 +29378,8 @@
       <c r="E607" s="1">
         <v>46054</v>
       </c>
-      <c r="F607" s="6" t="s">
-        <v>1395</v>
+      <c r="F607" t="s">
+        <v>126</v>
       </c>
       <c r="G607" t="s">
         <v>40</v>
@@ -29396,7 +29391,7 @@
         <v>70000</v>
       </c>
       <c r="O607" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
       <c r="P607">
         <v>3924</v>
@@ -29465,8 +29460,8 @@
       <c r="E609" s="1">
         <v>46054</v>
       </c>
-      <c r="F609" s="6" t="s">
-        <v>1396</v>
+      <c r="F609" t="s">
+        <v>34</v>
       </c>
       <c r="G609" t="s">
         <v>40</v>
@@ -29506,8 +29501,8 @@
       <c r="E610" s="1">
         <v>46054</v>
       </c>
-      <c r="F610" s="6" t="s">
-        <v>1396</v>
+      <c r="F610" t="s">
+        <v>34</v>
       </c>
       <c r="G610" t="s">
         <v>22</v>

</xml_diff>